<commit_message>
H ve DMT ile başlarsa tüketim değerini başka yerden al
</commit_message>
<xml_diff>
--- a/Faydalanma Atama/Faydalanma.xlsx
+++ b/Faydalanma Atama/Faydalanma.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yak\Desktop\Python\Faydalanma Atama\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B4754F20-6793-49CC-A067-5F92E8E3314E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E2DF172-BC34-4DDE-859B-4DBD974C7EE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="196">
   <si>
     <t>STATÜ KODU</t>
   </si>
@@ -58,25 +58,31 @@
     <t>FAYDALANMA BEKLİYOR</t>
   </si>
   <si>
-    <t>85370900-36</t>
-  </si>
-  <si>
-    <t>000000000040003333</t>
-  </si>
-  <si>
-    <t>TG 8.60MM-KT_C-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002291</t>
-  </si>
-  <si>
-    <t>TG 9.10MM-KT_B-83HC</t>
+    <t>69888400-22</t>
+  </si>
+  <si>
+    <t>000000000040002839</t>
+  </si>
+  <si>
+    <t>TV 1.30MM-70MC</t>
+  </si>
+  <si>
+    <t>000000000040002349</t>
+  </si>
+  <si>
+    <t>TV 1.70MM-45MC</t>
   </si>
   <si>
     <t>1385</t>
   </si>
   <si>
-    <t>68849900-87</t>
+    <t>68848800-181</t>
+  </si>
+  <si>
+    <t>000000000040002719</t>
+  </si>
+  <si>
+    <t>TG 3.30MM-KT_B-70MC</t>
   </si>
   <si>
     <t>000000000040002725</t>
@@ -85,58 +91,508 @@
     <t>TG 4.10MM-KT_AB-70MC</t>
   </si>
   <si>
+    <t>85961900-30</t>
+  </si>
+  <si>
+    <t>000000000040003138</t>
+  </si>
+  <si>
+    <t>TG 2.90MM-KT_AB-70MC</t>
+  </si>
+  <si>
+    <t>000000000040003137</t>
+  </si>
+  <si>
+    <t>TG 2.10MM-KT_AB-70MC</t>
+  </si>
+  <si>
+    <t>67307100-679</t>
+  </si>
+  <si>
+    <t>000000000040002428</t>
+  </si>
+  <si>
+    <t>TV 3.80MM-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002136</t>
+  </si>
+  <si>
+    <t>TF 5.50MM-70MC</t>
+  </si>
+  <si>
+    <t>68848700-6</t>
+  </si>
+  <si>
+    <t>000000000040002771</t>
+  </si>
+  <si>
+    <t>TG 3.10MM-KT_C-70MC</t>
+  </si>
+  <si>
+    <t>000000000040002172</t>
+  </si>
+  <si>
+    <t>TG 2.60MM-KT_AB-70MC</t>
+  </si>
+  <si>
+    <t>68848600-67</t>
+  </si>
+  <si>
+    <t>000000000040002770</t>
+  </si>
+  <si>
+    <t>TG 3.10MM-KT_C-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002737</t>
+  </si>
+  <si>
+    <t>TG 3.10MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002723</t>
+  </si>
+  <si>
+    <t>TG 3.60MM-KT_AB-70MC</t>
+  </si>
+  <si>
+    <t>68848200-265</t>
+  </si>
+  <si>
+    <t>000000000040002717</t>
+  </si>
+  <si>
+    <t>TG 3.10MM-KT_B-70MC</t>
+  </si>
+  <si>
+    <t>000000000040002248</t>
+  </si>
+  <si>
+    <t>TG 3.50MM-KT_B-75MC</t>
+  </si>
+  <si>
+    <t>67304500-290</t>
+  </si>
+  <si>
+    <t>000000000040002421</t>
+  </si>
+  <si>
+    <t>TV 2.80MM-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002378</t>
+  </si>
+  <si>
+    <t>TV 2.80MM-70MC</t>
+  </si>
+  <si>
+    <t>67305500-590</t>
+  </si>
+  <si>
+    <t>000000000040002402</t>
+  </si>
+  <si>
+    <t>TV 3.20MM-75MC</t>
+  </si>
+  <si>
+    <t>000000000040002424</t>
+  </si>
+  <si>
+    <t>TV 3.20MM-83HC</t>
+  </si>
+  <si>
+    <t>67305500-583</t>
+  </si>
+  <si>
+    <t>ycevik</t>
+  </si>
+  <si>
+    <t>70345500-326</t>
+  </si>
+  <si>
+    <t>000000000040002848</t>
+  </si>
+  <si>
+    <t>TG 2.90MM-KT_B-70MC</t>
+  </si>
+  <si>
+    <t>000000000040002716</t>
+  </si>
+  <si>
+    <t>TG 2.30MM-KT_AB-70MC</t>
+  </si>
+  <si>
+    <t>68851300-122</t>
+  </si>
+  <si>
+    <t>000000000040002746</t>
+  </si>
+  <si>
+    <t>TG 5.10MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002285</t>
+  </si>
+  <si>
+    <t>TG 5.60MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>67738000-630</t>
+  </si>
+  <si>
+    <t>000000000040002287</t>
+  </si>
+  <si>
+    <t>TG 6.10MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>67302400-521</t>
+  </si>
+  <si>
+    <t>000000000040002373</t>
+  </si>
+  <si>
+    <t>TV 2.20MM-70MC</t>
+  </si>
+  <si>
+    <t>000000000040002370</t>
+  </si>
+  <si>
+    <t>TV 1.80MM-70MC</t>
+  </si>
+  <si>
+    <t>67299400-35</t>
+  </si>
+  <si>
+    <t>000000000040002409</t>
+  </si>
+  <si>
+    <t>TV 1.40MM-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002367</t>
+  </si>
+  <si>
+    <t>TV 1.50MM-70MC</t>
+  </si>
+  <si>
+    <t>68848700-3</t>
+  </si>
+  <si>
+    <t>67302400-580</t>
+  </si>
+  <si>
+    <t>67304000-278</t>
+  </si>
+  <si>
+    <t>000000000040002400</t>
+  </si>
+  <si>
+    <t>TV 2.80MM-75MC</t>
+  </si>
+  <si>
+    <t>67305500-588</t>
+  </si>
+  <si>
+    <t>67307100-677</t>
+  </si>
+  <si>
+    <t>67306200-493</t>
+  </si>
+  <si>
+    <t>000000000040002426</t>
+  </si>
+  <si>
+    <t>TV 3.50MM-83HC</t>
+  </si>
+  <si>
+    <t>67738000-628</t>
+  </si>
+  <si>
+    <t>67307100-683</t>
+  </si>
+  <si>
+    <t>68850600-304</t>
+  </si>
+  <si>
+    <t>000000000040002726</t>
+  </si>
+  <si>
+    <t>TG 4.60MM-KT_B-70MC</t>
+  </si>
+  <si>
+    <t>000000000040002727</t>
+  </si>
+  <si>
+    <t>TG 4.60MM-KT_AB-70MC</t>
+  </si>
+  <si>
+    <t>67302400-590</t>
+  </si>
+  <si>
+    <t>sgarip</t>
+  </si>
+  <si>
+    <t>67302000-617</t>
+  </si>
+  <si>
+    <t>000000000040002372</t>
+  </si>
+  <si>
+    <t>TV 2.00MM-70MC</t>
+  </si>
+  <si>
+    <t>000000000040002376</t>
+  </si>
+  <si>
+    <t>TV 2.50MM-70MC</t>
+  </si>
+  <si>
+    <t>71707100-34</t>
+  </si>
+  <si>
+    <t>000000000040002924</t>
+  </si>
+  <si>
+    <t>TG 4.30MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>67305500-589</t>
+  </si>
+  <si>
+    <t>74002900-133</t>
+  </si>
+  <si>
+    <t>000000000040003023</t>
+  </si>
+  <si>
+    <t>TG 2.90MM-KT_B-75MC</t>
+  </si>
+  <si>
+    <t>67307000-44</t>
+  </si>
+  <si>
+    <t>000000000040002404</t>
+  </si>
+  <si>
+    <t>TV 3.80MM-75MC</t>
+  </si>
+  <si>
+    <t>000000000040002152</t>
+  </si>
+  <si>
+    <t>TF 5.50MM-83HC</t>
+  </si>
+  <si>
+    <t>67302500-245</t>
+  </si>
+  <si>
+    <t>000000000040002396</t>
+  </si>
+  <si>
+    <t>TV 2.20MM-75MC</t>
+  </si>
+  <si>
+    <t>68850600-305</t>
+  </si>
+  <si>
+    <t>70345500-330</t>
+  </si>
+  <si>
+    <t>67307100-681</t>
+  </si>
+  <si>
+    <t>80784000-75</t>
+  </si>
+  <si>
+    <t>000000000040003212</t>
+  </si>
+  <si>
+    <t>TG 3.30MM-KT_B-75MC</t>
+  </si>
+  <si>
+    <t>000000000040002722</t>
+  </si>
+  <si>
+    <t>TG 3.60MM-KT_B-70MC</t>
+  </si>
+  <si>
+    <t>86857800-17</t>
+  </si>
+  <si>
+    <t>000000000040003409</t>
+  </si>
+  <si>
+    <t>TV 5.30MM-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002339</t>
+  </si>
+  <si>
+    <t>TV 5.50MM-83HC</t>
+  </si>
+  <si>
+    <t>70345500-328</t>
+  </si>
+  <si>
+    <t>67307000-36</t>
+  </si>
+  <si>
+    <t>71673700-99</t>
+  </si>
+  <si>
+    <t>000000000040002922</t>
+  </si>
+  <si>
+    <t>TG 2.10MM-KT_B-70MC</t>
+  </si>
+  <si>
+    <t>000000000040002728</t>
+  </si>
+  <si>
+    <t>TG 1.85MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>67794200-1495</t>
+  </si>
+  <si>
+    <t>67305800-320</t>
+  </si>
+  <si>
+    <t>000000000040002381</t>
+  </si>
+  <si>
+    <t>TV 3.50MM-70MC</t>
+  </si>
+  <si>
+    <t>68848600-61</t>
+  </si>
+  <si>
+    <t>apankaduz</t>
+  </si>
+  <si>
+    <t>67303900-884</t>
+  </si>
+  <si>
+    <t>000000000040002380</t>
+  </si>
+  <si>
+    <t>TV 3.20MM-70MC</t>
+  </si>
+  <si>
+    <t>67308200-434</t>
+  </si>
+  <si>
+    <t>000000000040002431</t>
+  </si>
+  <si>
+    <t>TV 4.25MM-83HC</t>
+  </si>
+  <si>
+    <t>67301300-749</t>
+  </si>
+  <si>
+    <t>000000000040002371</t>
+  </si>
+  <si>
+    <t>TV 1.90MM-70MC</t>
+  </si>
+  <si>
+    <t>71673800-41</t>
+  </si>
+  <si>
+    <t>000000000040002923</t>
+  </si>
+  <si>
+    <t>TG 2.10MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>68849900-100</t>
+  </si>
+  <si>
     <t>000000000040002724</t>
   </si>
   <si>
     <t>TG 4.10MM-KT_B-70MC</t>
   </si>
   <si>
-    <t>68849900-152</t>
-  </si>
-  <si>
-    <t>67308200-417</t>
-  </si>
-  <si>
-    <t>000000000040002431</t>
-  </si>
-  <si>
-    <t>TV 4.25MM-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002428</t>
-  </si>
-  <si>
-    <t>TV 3.80MM-83HC</t>
-  </si>
-  <si>
-    <t>67302600-216</t>
-  </si>
-  <si>
-    <t>000000000040002417</t>
-  </si>
-  <si>
-    <t>TV 2.20MM-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002373</t>
-  </si>
-  <si>
-    <t>TV 2.20MM-70MC</t>
-  </si>
-  <si>
-    <t>67307800-495</t>
-  </si>
-  <si>
-    <t>000000000040002429</t>
-  </si>
-  <si>
-    <t>TV 4.00MM-83HC</t>
-  </si>
-  <si>
-    <t>sgarip</t>
-  </si>
-  <si>
-    <t>67303300-106</t>
+    <t>68850600-338</t>
+  </si>
+  <si>
+    <t>000000000040002741</t>
+  </si>
+  <si>
+    <t>TG 3.60MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002735</t>
+  </si>
+  <si>
+    <t>TG 2.90MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>68848600-30</t>
+  </si>
+  <si>
+    <t>67311600-142</t>
+  </si>
+  <si>
+    <t>000000000040002340</t>
+  </si>
+  <si>
+    <t>TV 6.50MM-83HC</t>
+  </si>
+  <si>
+    <t>000000000040002342</t>
+  </si>
+  <si>
+    <t>TV 8.00MM-83HC</t>
+  </si>
+  <si>
+    <t>67302500-261</t>
+  </si>
+  <si>
+    <t>67723500-263</t>
+  </si>
+  <si>
+    <t>000000000040002244</t>
+  </si>
+  <si>
+    <t>TG 2.60MM-KT_B-75MC</t>
+  </si>
+  <si>
+    <t>68850000-245</t>
+  </si>
+  <si>
+    <t>000000000040002743</t>
+  </si>
+  <si>
+    <t>TG 4.10MM-KT_B-83HC</t>
+  </si>
+  <si>
+    <t>68850600-337</t>
+  </si>
+  <si>
+    <t>68849900-99</t>
+  </si>
+  <si>
+    <t>71673700-98</t>
+  </si>
+  <si>
+    <t>68849500-95</t>
+  </si>
+  <si>
+    <t>000000000040002155</t>
+  </si>
+  <si>
+    <t>TF 7.00MM-83HC</t>
+  </si>
+  <si>
+    <t>67301300-750</t>
+  </si>
+  <si>
+    <t>67303300-125</t>
   </si>
   <si>
     <t>000000000040002398</t>
@@ -145,433 +601,13 @@
     <t>TV 2.50MM-75MC</t>
   </si>
   <si>
-    <t>67300500-143</t>
-  </si>
-  <si>
-    <t>000000000040002369</t>
-  </si>
-  <si>
-    <t>TV 1.65MM-70MC</t>
-  </si>
-  <si>
-    <t>000000000040002351</t>
-  </si>
-  <si>
-    <t>TV 2.00MM-45MC</t>
-  </si>
-  <si>
-    <t>67300500-145</t>
-  </si>
-  <si>
-    <t>000000000040002367</t>
-  </si>
-  <si>
-    <t>TV 1.50MM-70MC</t>
-  </si>
-  <si>
-    <t>67303900-873</t>
-  </si>
-  <si>
-    <t>000000000040002378</t>
-  </si>
-  <si>
-    <t>TV 2.80MM-70MC</t>
-  </si>
-  <si>
-    <t>67308200-380</t>
-  </si>
-  <si>
-    <t>000000000040002136</t>
-  </si>
-  <si>
-    <t>TF 5.50MM-70MC</t>
-  </si>
-  <si>
-    <t>67287699-775</t>
-  </si>
-  <si>
-    <t>000000000040002154</t>
-  </si>
-  <si>
-    <t>TF 6.50MM-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002699</t>
-  </si>
-  <si>
-    <t>PRV 6.50MM-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002152</t>
-  </si>
-  <si>
-    <t>TF 5.50MM-83HC</t>
-  </si>
-  <si>
-    <t>85370900-35</t>
-  </si>
-  <si>
-    <t>67305400-862</t>
-  </si>
-  <si>
-    <t>000000000040002380</t>
-  </si>
-  <si>
-    <t>TV 3.20MM-70MC</t>
-  </si>
-  <si>
-    <t>000000000040002376</t>
-  </si>
-  <si>
-    <t>TV 2.50MM-70MC</t>
-  </si>
-  <si>
-    <t>67300500-137</t>
-  </si>
-  <si>
-    <t>000000000040002370</t>
-  </si>
-  <si>
-    <t>TV 1.80MM-70MC</t>
-  </si>
-  <si>
-    <t>68848200-249</t>
-  </si>
-  <si>
-    <t>000000000040002717</t>
-  </si>
-  <si>
-    <t>TG 3.10MM-KT_B-70MC</t>
-  </si>
-  <si>
-    <t>000000000040002718</t>
-  </si>
-  <si>
-    <t>TG 3.10MM-KT_AB-70MC</t>
-  </si>
-  <si>
-    <t>67308800-369</t>
-  </si>
-  <si>
-    <t>000000000040002432</t>
-  </si>
-  <si>
-    <t>TV 4.50MM-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002434</t>
-  </si>
-  <si>
-    <t>TV 4.80MM-83HC</t>
-  </si>
-  <si>
-    <t>67300500-144</t>
-  </si>
-  <si>
-    <t>67303300-103</t>
-  </si>
-  <si>
-    <t>67794200-1476</t>
-  </si>
-  <si>
-    <t>67308200-414</t>
-  </si>
-  <si>
-    <t>000000000040002139</t>
-  </si>
-  <si>
-    <t>TF 5.50MM-75MC</t>
-  </si>
-  <si>
-    <t>67301300-604</t>
-  </si>
-  <si>
-    <t>000000000040002371</t>
-  </si>
-  <si>
-    <t>TV 1.90MM-70MC</t>
-  </si>
-  <si>
-    <t>apankaduz</t>
-  </si>
-  <si>
-    <t>67300500-146</t>
-  </si>
-  <si>
-    <t>67308200-418</t>
-  </si>
-  <si>
-    <t>67303300-109</t>
-  </si>
-  <si>
-    <t>68849400-236</t>
-  </si>
-  <si>
-    <t>000000000040002722</t>
-  </si>
-  <si>
-    <t>TG 3.60MM-KT_B-70MC</t>
-  </si>
-  <si>
-    <t>86857800-20</t>
-  </si>
-  <si>
-    <t>000000000040003409</t>
-  </si>
-  <si>
-    <t>TV 5.30MM-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002339</t>
-  </si>
-  <si>
-    <t>TV 5.50MM-83HC</t>
-  </si>
-  <si>
-    <t>85370900-15</t>
-  </si>
-  <si>
-    <t>68846800-212</t>
-  </si>
-  <si>
-    <t>000000000040002715</t>
-  </si>
-  <si>
-    <t>TG 2.30MM-KT_B-70MC</t>
-  </si>
-  <si>
-    <t>000000000040002922</t>
-  </si>
-  <si>
-    <t>TG 2.10MM-KT_B-70MC</t>
-  </si>
-  <si>
-    <t>67299700-219</t>
-  </si>
-  <si>
-    <t>000000000040002349</t>
-  </si>
-  <si>
-    <t>TV 1.70MM-45MC</t>
-  </si>
-  <si>
-    <t>67302000-594</t>
-  </si>
-  <si>
-    <t>000000000040002372</t>
-  </si>
-  <si>
-    <t>TV 2.00MM-70MC</t>
-  </si>
-  <si>
-    <t>000000000040002155</t>
-  </si>
-  <si>
-    <t>TF 7.00MM-83HC</t>
-  </si>
-  <si>
-    <t>67308200-415</t>
-  </si>
-  <si>
-    <t>68846800-213</t>
-  </si>
-  <si>
-    <t>68849900-154</t>
-  </si>
-  <si>
-    <t>67723300-28</t>
-  </si>
-  <si>
-    <t>000000000040002172</t>
-  </si>
-  <si>
-    <t>TG 2.60MM-KT_AB-70MC</t>
-  </si>
-  <si>
-    <t>000000000040002716</t>
-  </si>
-  <si>
-    <t>TG 2.30MM-KT_AB-70MC</t>
-  </si>
-  <si>
-    <t>000000000040002424</t>
-  </si>
-  <si>
-    <t>TV 3.20MM-83HC</t>
-  </si>
-  <si>
-    <t>67302400-530</t>
-  </si>
-  <si>
-    <t>000000000040002414</t>
-  </si>
-  <si>
-    <t>TV 1.80MM-83HC</t>
-  </si>
-  <si>
-    <t>68850900-159</t>
-  </si>
-  <si>
-    <t>000000000040002735</t>
-  </si>
-  <si>
-    <t>TG 2.90MM-KT_B-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002739</t>
-  </si>
-  <si>
-    <t>TG 3.30MM-KT_B-83HC</t>
-  </si>
-  <si>
-    <t>67302600-217</t>
-  </si>
-  <si>
-    <t>67307500-392</t>
-  </si>
-  <si>
-    <t>000000000040002383</t>
-  </si>
-  <si>
-    <t>TV 4.00MM-70MC</t>
-  </si>
-  <si>
-    <t>67308800-371</t>
-  </si>
-  <si>
-    <t>67739500-178</t>
-  </si>
-  <si>
-    <t>000000000040002289</t>
-  </si>
-  <si>
-    <t>TG 7.10MM-KT_B-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002292</t>
-  </si>
-  <si>
-    <t>TG 10.10MM-KT_B-83HC</t>
-  </si>
-  <si>
-    <t>86154800-5</t>
-  </si>
-  <si>
-    <t>000000000040003371</t>
-  </si>
-  <si>
-    <t>TG 7.10MM-KT_C-70MC</t>
-  </si>
-  <si>
-    <t>85370900-37</t>
-  </si>
-  <si>
-    <t>86857800-15</t>
-  </si>
-  <si>
-    <t>ycevik</t>
-  </si>
-  <si>
-    <t>87430500-1</t>
-  </si>
-  <si>
-    <t>000000000040003449</t>
-  </si>
-  <si>
-    <t>TG 4.60MM-KT_C-75MC</t>
-  </si>
-  <si>
-    <t>000000000040002776</t>
-  </si>
-  <si>
-    <t>TG 4.60MM-KT_C-70MC</t>
-  </si>
-  <si>
-    <t>85370900-11</t>
-  </si>
-  <si>
-    <t>67303300-111</t>
-  </si>
-  <si>
-    <t>67307800-496</t>
-  </si>
-  <si>
-    <t>68847000-110</t>
-  </si>
-  <si>
-    <t>000000000040002732</t>
-  </si>
-  <si>
-    <t>TG 2.30MM-KT_B-83HC</t>
-  </si>
-  <si>
-    <t>68849900-129</t>
-  </si>
-  <si>
-    <t>79559900-28</t>
-  </si>
-  <si>
-    <t>000000000040002416</t>
-  </si>
-  <si>
-    <t>TV 2.00MM-83HC</t>
-  </si>
-  <si>
-    <t>79559900-30</t>
-  </si>
-  <si>
-    <t>67302400-524</t>
-  </si>
-  <si>
-    <t>67737300-159</t>
-  </si>
-  <si>
-    <t>000000000040002181</t>
-  </si>
-  <si>
-    <t>TG 5.60MM-KT_AB-70MC</t>
-  </si>
-  <si>
-    <t>000000000040002231</t>
-  </si>
-  <si>
-    <t>TG 5.60MM-KT_B-70MC</t>
-  </si>
-  <si>
-    <t>67308200-416</t>
-  </si>
-  <si>
-    <t>85370900-13</t>
-  </si>
-  <si>
-    <t>85370900-26</t>
-  </si>
-  <si>
-    <t>85362500-23</t>
-  </si>
-  <si>
-    <t>000000000040003332</t>
-  </si>
-  <si>
-    <t>TG 8.10MM-KT_C-83HC</t>
-  </si>
-  <si>
-    <t>67729800-6</t>
-  </si>
-  <si>
-    <t>000000000040002327</t>
-  </si>
-  <si>
-    <t>TG 4.60MM-KT_C-83HC</t>
-  </si>
-  <si>
-    <t>000000000040002281</t>
-  </si>
-  <si>
-    <t>TG 4.60MM-KT_B-83HC</t>
-  </si>
-  <si>
-    <t>67723300-63</t>
+    <t>67794200-1507</t>
+  </si>
+  <si>
+    <t>68850000-246</t>
+  </si>
+  <si>
+    <t>67794200-1494</t>
   </si>
 </sst>
 </file>
@@ -616,7 +652,7 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{93DC0BEB-F587-4E36-9E57-6A537FBF7D96}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{9DFCCFAA-58F2-4D27-A5A2-1446D1298631}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -630,8 +666,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K81">
-  <autoFilter ref="A1:K81" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K92">
+  <autoFilter ref="A1:K92" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="STATÜ KODU"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="BARKOD NUMARASI"/>
@@ -966,7 +1002,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="9.140625" style="1" customWidth="1"/>
@@ -1022,7 +1058,7 @@
         <v>14</v>
       </c>
       <c r="E2">
-        <v>862151</v>
+        <v>863689</v>
       </c>
       <c r="F2" t="s">
         <v>15</v>
@@ -1031,10 +1067,10 @@
         <v>16</v>
       </c>
       <c r="H2">
-        <v>3421</v>
+        <v>19721.257692307699</v>
       </c>
       <c r="I2" s="1">
-        <v>46013.352488425902</v>
+        <v>46027.377592592602</v>
       </c>
       <c r="J2" t="s">
         <v>17</v>
@@ -1054,7 +1090,7 @@
         <v>20</v>
       </c>
       <c r="E3">
-        <v>872888</v>
+        <v>877115</v>
       </c>
       <c r="F3" t="s">
         <v>21</v>
@@ -1063,10 +1099,10 @@
         <v>22</v>
       </c>
       <c r="H3">
-        <v>3638.43</v>
+        <v>4091.3609090909104</v>
       </c>
       <c r="I3" s="1">
-        <v>46013.395219907397</v>
+        <v>46027.3989351852</v>
       </c>
       <c r="J3" t="s">
         <v>17</v>
@@ -1080,25 +1116,25 @@
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E4">
-        <v>872773</v>
+        <v>877116</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="H4">
-        <v>11101</v>
+        <v>3649.6325048170002</v>
       </c>
       <c r="I4" s="1">
-        <v>46013.395648148202</v>
+        <v>46027.402731481503</v>
       </c>
       <c r="J4" t="s">
         <v>17</v>
@@ -1109,28 +1145,28 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E5">
-        <v>865310</v>
+        <v>877555</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H5">
-        <v>7451</v>
+        <v>10438.047138047101</v>
       </c>
       <c r="I5" s="1">
-        <v>46013.413240740701</v>
+        <v>46027.407766203702</v>
       </c>
       <c r="J5" t="s">
         <v>17</v>
@@ -1141,28 +1177,28 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E6">
-        <v>872367</v>
+        <v>877659</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H6">
-        <v>20402</v>
+        <v>11313.8643676223</v>
       </c>
       <c r="I6" s="1">
-        <v>46013.415300925903</v>
+        <v>46027.408171296302</v>
       </c>
       <c r="J6" t="s">
         <v>17</v>
@@ -1173,31 +1209,31 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E7">
-        <v>865277</v>
+        <v>877951</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="H7">
-        <v>7586.5300000000007</v>
+        <v>6194.2075042158503</v>
       </c>
       <c r="I7" s="1">
-        <v>46013.448171296302</v>
+        <v>46027.408715277801</v>
       </c>
       <c r="J7" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1205,28 +1241,28 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E8">
-        <v>872367</v>
+        <v>877117</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="G8" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="H8">
-        <v>10363</v>
+        <v>2004.23090909091</v>
       </c>
       <c r="I8" s="1">
-        <v>46013.448229166701</v>
+        <v>46027.410740740699</v>
       </c>
       <c r="J8" t="s">
         <v>17</v>
@@ -1237,31 +1273,31 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="E9">
-        <v>864964</v>
+        <v>877117</v>
       </c>
       <c r="F9" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="G9" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="H9">
-        <v>7379.01</v>
+        <v>8104.2616216216193</v>
       </c>
       <c r="I9" s="1">
-        <v>46013.452025462997</v>
+        <v>46027.415115740703</v>
       </c>
       <c r="J9" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1269,28 +1305,28 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="D10" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="E10">
-        <v>870932</v>
+        <v>863677</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="G10" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="H10">
-        <v>7973.9199999999801</v>
+        <v>8330.4886776860003</v>
       </c>
       <c r="I10" s="1">
-        <v>46013.479212963</v>
+        <v>46027.418148148201</v>
       </c>
       <c r="J10" t="s">
         <v>17</v>
@@ -1301,28 +1337,28 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="D11" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="E11">
-        <v>872363</v>
+        <v>865047</v>
       </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G11" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="H11">
-        <v>28274</v>
+        <v>2766.4721518986998</v>
       </c>
       <c r="I11" s="1">
-        <v>46013.479409722197</v>
+        <v>46027.444247685198</v>
       </c>
       <c r="J11" t="s">
         <v>17</v>
@@ -1333,31 +1369,31 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E12">
-        <v>872367</v>
+        <v>877426</v>
       </c>
       <c r="F12" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="G12" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="H12">
-        <v>11134.08</v>
+        <v>6749.13278481013</v>
       </c>
       <c r="I12" s="1">
-        <v>46013.523564814801</v>
+        <v>46027.4468402778</v>
       </c>
       <c r="J12" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1365,31 +1401,31 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="E13">
-        <v>872109</v>
+        <v>877722</v>
       </c>
       <c r="F13" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="G13" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H13">
-        <v>3973.38</v>
+        <v>5411.1688631984998</v>
       </c>
       <c r="I13" s="1">
-        <v>46013.531145833302</v>
+        <v>46027.458923611099</v>
       </c>
       <c r="J13" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1397,31 +1433,31 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E14">
-        <v>849200</v>
+        <v>878413</v>
       </c>
       <c r="F14" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="G14" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="H14">
-        <v>7804</v>
+        <v>2556.1097256857902</v>
       </c>
       <c r="I14" s="1">
-        <v>46013.5316087963</v>
+        <v>46027.475046296298</v>
       </c>
       <c r="J14" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1429,31 +1465,31 @@
         <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C15" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="E15">
-        <v>871265</v>
+        <v>878271</v>
       </c>
       <c r="F15" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="G15" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="H15">
-        <v>3010.53</v>
+        <v>1264.9871975180999</v>
       </c>
       <c r="I15" s="1">
-        <v>46013.534293981502</v>
+        <v>46027.475277777798</v>
       </c>
       <c r="J15" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1461,28 +1497,28 @@
         <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>76</v>
       </c>
       <c r="D16" t="s">
-        <v>14</v>
+        <v>77</v>
       </c>
       <c r="E16">
-        <v>862151</v>
+        <v>864268</v>
       </c>
       <c r="F16" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="G16" t="s">
-        <v>16</v>
+        <v>79</v>
       </c>
       <c r="H16">
-        <v>3427</v>
+        <v>18461.538461538501</v>
       </c>
       <c r="I16" s="1">
-        <v>46013.535601851901</v>
+        <v>46027.479421296302</v>
       </c>
       <c r="J16" t="s">
         <v>17</v>
@@ -1493,28 +1529,28 @@
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="D17" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="E17">
-        <v>872410</v>
+        <v>864272</v>
       </c>
       <c r="F17" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="G17" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="H17">
-        <v>9962.2999999999993</v>
+        <v>22809.917355371901</v>
       </c>
       <c r="I17" s="1">
-        <v>46013.542569444398</v>
+        <v>46027.479699074102</v>
       </c>
       <c r="J17" t="s">
         <v>17</v>
@@ -1525,31 +1561,31 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E18">
-        <v>872359</v>
+        <v>877943</v>
       </c>
       <c r="F18" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="G18" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="H18">
-        <v>4006.4966666667001</v>
+        <v>12512.647554806101</v>
       </c>
       <c r="I18" s="1">
-        <v>46013.544085648202</v>
+        <v>46027.528692129599</v>
       </c>
       <c r="J18" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -1557,28 +1593,28 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E19">
-        <v>872826</v>
+        <v>877717</v>
       </c>
       <c r="F19" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="G19" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="H19">
-        <v>3232.08</v>
+        <v>4012.9588631984998</v>
       </c>
       <c r="I19" s="1">
-        <v>46013.586087962998</v>
+        <v>46027.541122685201</v>
       </c>
       <c r="J19" t="s">
         <v>17</v>
@@ -1589,28 +1625,28 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" t="s">
         <v>76</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>77</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20">
+        <v>863659</v>
+      </c>
+      <c r="F20" t="s">
         <v>78</v>
       </c>
-      <c r="E20">
-        <v>868554</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>79</v>
       </c>
-      <c r="G20" t="s">
-        <v>80</v>
-      </c>
       <c r="H20">
-        <v>5685</v>
+        <v>6527.2371906355002</v>
       </c>
       <c r="I20" s="1">
-        <v>46013.586666666699</v>
+        <v>46027.541469907403</v>
       </c>
       <c r="J20" t="s">
         <v>17</v>
@@ -1621,28 +1657,28 @@
         <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="D21" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="E21">
-        <v>872346</v>
+        <v>874027</v>
       </c>
       <c r="F21" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G21" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H21">
-        <v>29167</v>
+        <v>15409.3056198347</v>
       </c>
       <c r="I21" s="1">
-        <v>46013.623645833301</v>
+        <v>46027.541898148098</v>
       </c>
       <c r="J21" t="s">
         <v>17</v>
@@ -1653,28 +1689,28 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="D22" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="E22">
-        <v>865306</v>
+        <v>865047</v>
       </c>
       <c r="F22" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="G22" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H22">
-        <v>3823.09</v>
+        <v>14715.9810126582</v>
       </c>
       <c r="I22" s="1">
-        <v>46013.6263078704</v>
+        <v>46027.548912036997</v>
       </c>
       <c r="J22" t="s">
         <v>17</v>
@@ -1685,28 +1721,28 @@
         <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="D23" t="s">
-        <v>67</v>
+        <v>30</v>
       </c>
       <c r="E23">
-        <v>872139</v>
+        <v>877310</v>
       </c>
       <c r="F23" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="G23" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H23">
-        <v>8537.5400000000009</v>
+        <v>11582.491582491601</v>
       </c>
       <c r="I23" s="1">
-        <v>46013.637685185196</v>
+        <v>46027.5559490741</v>
       </c>
       <c r="J23" t="s">
         <v>17</v>
@@ -1717,31 +1753,31 @@
         <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="D24" t="s">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="E24">
-        <v>872143</v>
+        <v>864288</v>
       </c>
       <c r="F24" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="G24" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="H24">
-        <v>8241</v>
+        <v>6414.1171906355003</v>
       </c>
       <c r="I24" s="1">
-        <v>46013.648587962998</v>
+        <v>46027.556284722203</v>
       </c>
       <c r="J24" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -1749,31 +1785,31 @@
         <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C25" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D25" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E25">
-        <v>870932</v>
+        <v>877463</v>
       </c>
       <c r="F25" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="G25" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="H25">
-        <v>8830.7526457398999</v>
+        <v>4432.2234391534002</v>
       </c>
       <c r="I25" s="1">
-        <v>46013.687280092599</v>
+        <v>46027.6086111111</v>
       </c>
       <c r="J25" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -1781,31 +1817,31 @@
         <v>11</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="D26" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="E26">
-        <v>872359</v>
+        <v>878223</v>
       </c>
       <c r="F26" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G26" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="H26">
-        <v>5358</v>
+        <v>8505.6876938986607</v>
       </c>
       <c r="I26" s="1">
-        <v>46013.694525462997</v>
+        <v>46027.608912037002</v>
       </c>
       <c r="J26" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -1813,31 +1849,31 @@
         <v>11</v>
       </c>
       <c r="B27" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C27" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D27" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E27">
-        <v>865257</v>
+        <v>877555</v>
       </c>
       <c r="F27" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G27" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H27">
-        <v>7765</v>
+        <v>10190.7968574635</v>
       </c>
       <c r="I27" s="1">
-        <v>46013.720648148097</v>
+        <v>46027.622048611098</v>
       </c>
       <c r="J27" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -1845,31 +1881,31 @@
         <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C28" t="s">
-        <v>39</v>
+        <v>98</v>
       </c>
       <c r="D28" t="s">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="E28">
-        <v>865306</v>
+        <v>874127</v>
       </c>
       <c r="F28" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G28" t="s">
-        <v>51</v>
+        <v>101</v>
       </c>
       <c r="H28">
-        <v>14508</v>
+        <v>3602</v>
       </c>
       <c r="I28" s="1">
-        <v>46013.721261574101</v>
+        <v>46027.633379629602</v>
       </c>
       <c r="J28" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -1877,31 +1913,31 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C29" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="D29" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="E29">
-        <v>872826</v>
+        <v>864264</v>
       </c>
       <c r="F29" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G29" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H29">
-        <v>4627.04</v>
+        <v>15919.7324414716</v>
       </c>
       <c r="I29" s="1">
-        <v>46013.729513888902</v>
+        <v>46027.685370370396</v>
       </c>
       <c r="J29" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -1909,31 +1945,31 @@
         <v>11</v>
       </c>
       <c r="B30" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D30" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="E30">
-        <v>871980</v>
+        <v>863685</v>
       </c>
       <c r="F30" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="G30" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="H30">
-        <v>5000.4399999999996</v>
+        <v>4844.72</v>
       </c>
       <c r="I30" s="1">
-        <v>46013.742337962998</v>
+        <v>46027.688726851899</v>
       </c>
       <c r="J30" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -1941,31 +1977,31 @@
         <v>11</v>
       </c>
       <c r="B31" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="C31" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="D31" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="E31">
-        <v>862151</v>
+        <v>863672</v>
       </c>
       <c r="F31" t="s">
-        <v>15</v>
+        <v>83</v>
       </c>
       <c r="G31" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="H31">
-        <v>4188.0070160052601</v>
+        <v>21714.2873553719</v>
       </c>
       <c r="I31" s="1">
-        <v>46013.7519791667</v>
+        <v>46027.689062500001</v>
       </c>
       <c r="J31" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -1973,31 +2009,31 @@
         <v>11</v>
       </c>
       <c r="B32" t="s">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="C32" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="D32" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E32">
-        <v>872810</v>
+        <v>841399</v>
       </c>
       <c r="F32" t="s">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="G32" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="H32">
-        <v>2424.0300000000002</v>
+        <v>5251.4971906355004</v>
       </c>
       <c r="I32" s="1">
-        <v>46013.752511574101</v>
+        <v>46027.694247685198</v>
       </c>
       <c r="J32" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -2005,31 +2041,31 @@
         <v>11</v>
       </c>
       <c r="B33" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33">
+        <v>868353</v>
+      </c>
+      <c r="F33" t="s">
+        <v>107</v>
+      </c>
+      <c r="G33" t="s">
+        <v>108</v>
+      </c>
+      <c r="H33">
+        <v>11534.1410126582</v>
+      </c>
+      <c r="I33" s="1">
+        <v>46027.706041666701</v>
+      </c>
+      <c r="J33" t="s">
         <v>103</v>
-      </c>
-      <c r="C33" t="s">
-        <v>104</v>
-      </c>
-      <c r="D33" t="s">
-        <v>105</v>
-      </c>
-      <c r="E33">
-        <v>872892</v>
-      </c>
-      <c r="F33" t="s">
-        <v>106</v>
-      </c>
-      <c r="G33" t="s">
-        <v>107</v>
-      </c>
-      <c r="H33">
-        <v>308.84999999999599</v>
-      </c>
-      <c r="I33" s="1">
-        <v>46013.779861111099</v>
-      </c>
-      <c r="J33" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -2037,31 +2073,31 @@
         <v>11</v>
       </c>
       <c r="B34" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C34" t="s">
-        <v>47</v>
+        <v>110</v>
       </c>
       <c r="D34" t="s">
-        <v>48</v>
+        <v>111</v>
       </c>
       <c r="E34">
-        <v>871907</v>
+        <v>874127</v>
       </c>
       <c r="F34" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="G34" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="H34">
-        <v>35972</v>
+        <v>5264</v>
       </c>
       <c r="I34" s="1">
-        <v>46013.789212962998</v>
+        <v>46027.707511574103</v>
       </c>
       <c r="J34" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -2069,31 +2105,31 @@
         <v>11</v>
       </c>
       <c r="B35" t="s">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="C35" t="s">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="D35" t="s">
-        <v>113</v>
+        <v>57</v>
       </c>
       <c r="E35">
-        <v>874072</v>
+        <v>868362</v>
       </c>
       <c r="F35" t="s">
-        <v>69</v>
+        <v>107</v>
       </c>
       <c r="G35" t="s">
-        <v>70</v>
+        <v>108</v>
       </c>
       <c r="H35">
-        <v>7086</v>
+        <v>10139.8410126582</v>
       </c>
       <c r="I35" s="1">
-        <v>46013.7896064815</v>
+        <v>46027.710277777798</v>
       </c>
       <c r="J35" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -2101,31 +2137,31 @@
         <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="C36" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="D36" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="E36">
-        <v>866835</v>
+        <v>877635</v>
       </c>
       <c r="F36" t="s">
-        <v>114</v>
+        <v>31</v>
       </c>
       <c r="G36" t="s">
-        <v>115</v>
+        <v>32</v>
       </c>
       <c r="H36">
-        <v>3965.05</v>
+        <v>2714.6668574635</v>
       </c>
       <c r="I36" s="1">
-        <v>46013.791412036997</v>
+        <v>46027.769131944398</v>
       </c>
       <c r="J36" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -2133,31 +2169,31 @@
         <v>11</v>
       </c>
       <c r="B37" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="C37" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="D37" t="s">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="E37">
-        <v>864964</v>
+        <v>841390</v>
       </c>
       <c r="F37" t="s">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="G37" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="H37">
-        <v>8133</v>
+        <v>14554.422441471601</v>
       </c>
       <c r="I37" s="1">
-        <v>46013.791817129597</v>
+        <v>46027.769432870402</v>
       </c>
       <c r="J37" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -2165,31 +2201,31 @@
         <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>117</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="D38" t="s">
-        <v>105</v>
+        <v>57</v>
       </c>
       <c r="E38">
-        <v>872892</v>
+        <v>874049</v>
       </c>
       <c r="F38" t="s">
-        <v>106</v>
+        <v>53</v>
       </c>
       <c r="G38" t="s">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="H38">
-        <v>14571</v>
+        <v>7526.5610126581996</v>
       </c>
       <c r="I38" s="1">
-        <v>46013.8210763889</v>
+        <v>46027.769699074102</v>
       </c>
       <c r="J38" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
@@ -2197,31 +2233,31 @@
         <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C39" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="D39" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="E39">
-        <v>872773</v>
+        <v>874049</v>
       </c>
       <c r="F39" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="G39" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="H39">
-        <v>9170</v>
+        <v>12120.253164557</v>
       </c>
       <c r="I39" s="1">
-        <v>46013.821921296301</v>
+        <v>46027.787048611099</v>
       </c>
       <c r="J39" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
@@ -2229,31 +2265,31 @@
         <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>119</v>
+        <v>62</v>
       </c>
       <c r="C40" t="s">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="D40" t="s">
-        <v>121</v>
+        <v>64</v>
       </c>
       <c r="E40">
-        <v>872854</v>
+        <v>878085</v>
       </c>
       <c r="F40" t="s">
-        <v>122</v>
+        <v>65</v>
       </c>
       <c r="G40" t="s">
-        <v>123</v>
+        <v>66</v>
       </c>
       <c r="H40">
-        <v>15588</v>
+        <v>2515.1188631985001</v>
       </c>
       <c r="I40" s="1">
-        <v>46013.822916666701</v>
+        <v>46027.805381944403</v>
       </c>
       <c r="J40" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
@@ -2261,31 +2297,31 @@
         <v>11</v>
       </c>
       <c r="B41" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="C41" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="D41" t="s">
-        <v>51</v>
+        <v>115</v>
       </c>
       <c r="E41">
-        <v>866496</v>
+        <v>878085</v>
       </c>
       <c r="F41" t="s">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="G41" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="H41">
-        <v>8564.43</v>
+        <v>9456.3409248554999</v>
       </c>
       <c r="I41" s="1">
-        <v>46013.829560185201</v>
+        <v>46027.805775462999</v>
       </c>
       <c r="J41" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -2293,31 +2329,31 @@
         <v>11</v>
       </c>
       <c r="B42" t="s">
-        <v>83</v>
+        <v>116</v>
       </c>
       <c r="C42" t="s">
-        <v>66</v>
+        <v>117</v>
       </c>
       <c r="D42" t="s">
-        <v>67</v>
+        <v>118</v>
       </c>
       <c r="E42">
-        <v>874076</v>
+        <v>877635</v>
       </c>
       <c r="F42" t="s">
-        <v>124</v>
+        <v>31</v>
       </c>
       <c r="G42" t="s">
-        <v>125</v>
+        <v>32</v>
       </c>
       <c r="H42">
-        <v>3456.73</v>
+        <v>3187.4298540965201</v>
       </c>
       <c r="I42" s="1">
-        <v>46013.849085648202</v>
+        <v>46027.808958333299</v>
       </c>
       <c r="J42" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -2325,31 +2361,31 @@
         <v>11</v>
       </c>
       <c r="B43" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D43" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E43">
-        <v>871275</v>
+        <v>674060</v>
       </c>
       <c r="F43" t="s">
-        <v>50</v>
+        <v>119</v>
       </c>
       <c r="G43" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="H43">
-        <v>8167.17</v>
+        <v>9329.2015824915998</v>
       </c>
       <c r="I43" s="1">
-        <v>46013.878819444399</v>
+        <v>46027.809837963003</v>
       </c>
       <c r="J43" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -2357,31 +2393,31 @@
         <v>11</v>
       </c>
       <c r="B44" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C44" t="s">
-        <v>32</v>
+        <v>122</v>
       </c>
       <c r="D44" t="s">
-        <v>33</v>
+        <v>123</v>
       </c>
       <c r="E44">
-        <v>874073</v>
+        <v>864130</v>
       </c>
       <c r="F44" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="G44" t="s">
-        <v>128</v>
+        <v>108</v>
       </c>
       <c r="H44">
-        <v>13211</v>
+        <v>10353.730602006701</v>
       </c>
       <c r="I44" s="1">
-        <v>46013.8901273148</v>
+        <v>46027.828865740703</v>
       </c>
       <c r="J44" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -2389,31 +2425,31 @@
         <v>11</v>
       </c>
       <c r="B45" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C45" t="s">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="D45" t="s">
-        <v>131</v>
+        <v>99</v>
       </c>
       <c r="E45">
-        <v>865583</v>
+        <v>874127</v>
       </c>
       <c r="F45" t="s">
-        <v>132</v>
+        <v>100</v>
       </c>
       <c r="G45" t="s">
-        <v>133</v>
+        <v>101</v>
       </c>
       <c r="H45">
-        <v>14105</v>
+        <v>5119</v>
       </c>
       <c r="I45" s="1">
-        <v>46013.8907175926</v>
+        <v>46027.878171296303</v>
       </c>
       <c r="J45" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
@@ -2421,31 +2457,31 @@
         <v>11</v>
       </c>
       <c r="B46" t="s">
-        <v>49</v>
+        <v>125</v>
       </c>
       <c r="C46" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="D46" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="E46">
-        <v>871383</v>
+        <v>877734</v>
       </c>
       <c r="F46" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="G46" t="s">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="H46">
-        <v>6084.78</v>
+        <v>5926.8895375722996</v>
       </c>
       <c r="I46" s="1">
-        <v>46013.897071759297</v>
+        <v>46027.888495370396</v>
       </c>
       <c r="J46" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
@@ -2453,31 +2489,31 @@
         <v>11</v>
       </c>
       <c r="B47" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C47" t="s">
+        <v>29</v>
+      </c>
+      <c r="D47" t="s">
         <v>30</v>
       </c>
-      <c r="D47" t="s">
-        <v>31</v>
-      </c>
       <c r="E47">
-        <v>872367</v>
+        <v>877310</v>
       </c>
       <c r="F47" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="G47" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="H47">
-        <v>15552</v>
+        <v>11492.7048260382</v>
       </c>
       <c r="I47" s="1">
-        <v>46013.8975810185</v>
+        <v>46027.888819444401</v>
       </c>
       <c r="J47" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -2485,31 +2521,31 @@
         <v>11</v>
       </c>
       <c r="B48" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C48" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D48" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="E48">
-        <v>864701</v>
+        <v>877576</v>
       </c>
       <c r="F48" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="G48" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="H48">
-        <v>8106</v>
+        <v>1904.7619047619</v>
       </c>
       <c r="I48" s="1">
-        <v>46013.898043981499</v>
+        <v>46027.889444444401</v>
       </c>
       <c r="J48" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
@@ -2517,31 +2553,31 @@
         <v>11</v>
       </c>
       <c r="B49" t="s">
-        <v>92</v>
+        <v>132</v>
       </c>
       <c r="C49" t="s">
-        <v>25</v>
+        <v>133</v>
       </c>
       <c r="D49" t="s">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="E49">
-        <v>864701</v>
+        <v>878867</v>
       </c>
       <c r="F49" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="G49" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="H49">
-        <v>623.55999999999904</v>
+        <v>14414.4696505212</v>
       </c>
       <c r="I49" s="1">
-        <v>46013.898472222201</v>
+        <v>46027.889872685198</v>
       </c>
       <c r="J49" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
@@ -2549,31 +2585,31 @@
         <v>11</v>
       </c>
       <c r="B50" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C50" t="s">
-        <v>136</v>
+        <v>63</v>
       </c>
       <c r="D50" t="s">
-        <v>137</v>
+        <v>64</v>
       </c>
       <c r="E50">
-        <v>864717</v>
+        <v>878085</v>
       </c>
       <c r="F50" t="s">
-        <v>124</v>
+        <v>65</v>
       </c>
       <c r="G50" t="s">
-        <v>125</v>
+        <v>66</v>
       </c>
       <c r="H50">
-        <v>7113.75</v>
+        <v>16763.005780346801</v>
       </c>
       <c r="I50" s="1">
-        <v>46013.904976851903</v>
+        <v>46027.891180555598</v>
       </c>
       <c r="J50" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
@@ -2584,28 +2620,28 @@
         <v>138</v>
       </c>
       <c r="C51" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="D51" t="s">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="E51">
-        <v>868554</v>
+        <v>877635</v>
       </c>
       <c r="F51" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="G51" t="s">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="H51">
-        <v>6966</v>
+        <v>4017.95735129068</v>
       </c>
       <c r="I51" s="1">
-        <v>46013.908587963</v>
+        <v>46027.908657407403</v>
       </c>
       <c r="J51" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
@@ -2613,31 +2649,31 @@
         <v>11</v>
       </c>
       <c r="B52" t="s">
+        <v>127</v>
+      </c>
+      <c r="C52" t="s">
+        <v>128</v>
+      </c>
+      <c r="D52" t="s">
         <v>129</v>
       </c>
-      <c r="C52" t="s">
+      <c r="E52">
+        <v>877616</v>
+      </c>
+      <c r="F52" t="s">
         <v>130</v>
       </c>
-      <c r="D52" t="s">
+      <c r="G52" t="s">
         <v>131</v>
       </c>
-      <c r="E52">
-        <v>865542</v>
-      </c>
-      <c r="F52" t="s">
-        <v>132</v>
-      </c>
-      <c r="G52" t="s">
-        <v>133</v>
-      </c>
       <c r="H52">
-        <v>11110.06</v>
+        <v>912.17190476190001</v>
       </c>
       <c r="I52" s="1">
-        <v>46013.917476851799</v>
+        <v>46027.916620370401</v>
       </c>
       <c r="J52" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
@@ -2645,31 +2681,31 @@
         <v>11</v>
       </c>
       <c r="B53" t="s">
-        <v>126</v>
+        <v>95</v>
       </c>
       <c r="C53" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="D53" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="E53">
-        <v>871942</v>
+        <v>878405</v>
       </c>
       <c r="F53" t="s">
-        <v>127</v>
+        <v>73</v>
       </c>
       <c r="G53" t="s">
-        <v>128</v>
+        <v>74</v>
       </c>
       <c r="H53">
-        <v>12713.4</v>
+        <v>7210.3176938986599</v>
       </c>
       <c r="I53" s="1">
-        <v>46013.918020833298</v>
+        <v>46027.947106481501</v>
       </c>
       <c r="J53" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
@@ -2686,7 +2722,7 @@
         <v>141</v>
       </c>
       <c r="E54">
-        <v>870964</v>
+        <v>877540</v>
       </c>
       <c r="F54" t="s">
         <v>142</v>
@@ -2695,13 +2731,13 @@
         <v>143</v>
       </c>
       <c r="H54">
-        <v>1402.8314028314001</v>
+        <v>27426.470588235301</v>
       </c>
       <c r="I54" s="1">
-        <v>46013.927407407398</v>
+        <v>46027.948923611097</v>
       </c>
       <c r="J54" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
@@ -2712,28 +2748,28 @@
         <v>144</v>
       </c>
       <c r="C55" t="s">
-        <v>145</v>
+        <v>107</v>
       </c>
       <c r="D55" t="s">
-        <v>146</v>
+        <v>108</v>
       </c>
       <c r="E55">
-        <v>870964</v>
+        <v>841381</v>
       </c>
       <c r="F55" t="s">
-        <v>142</v>
+        <v>76</v>
       </c>
       <c r="G55" t="s">
-        <v>143</v>
+        <v>77</v>
       </c>
       <c r="H55">
-        <v>1685.06223938224</v>
+        <v>21088.0829015544</v>
       </c>
       <c r="I55" s="1">
-        <v>46013.929085648102</v>
+        <v>46027.952708333301</v>
       </c>
       <c r="J55" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
@@ -2741,31 +2777,31 @@
         <v>11</v>
       </c>
       <c r="B56" t="s">
-        <v>147</v>
+        <v>95</v>
       </c>
       <c r="C56" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="D56" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="E56">
-        <v>862151</v>
+        <v>878455</v>
       </c>
       <c r="F56" t="s">
-        <v>15</v>
+        <v>73</v>
       </c>
       <c r="G56" t="s">
-        <v>16</v>
+        <v>74</v>
       </c>
       <c r="H56">
-        <v>5263</v>
+        <v>7059.4276938986604</v>
       </c>
       <c r="I56" s="1">
-        <v>46013.9469328704</v>
+        <v>46027.955462963</v>
       </c>
       <c r="J56" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
@@ -2773,31 +2809,31 @@
         <v>11</v>
       </c>
       <c r="B57" t="s">
-        <v>116</v>
+        <v>145</v>
       </c>
       <c r="C57" t="s">
-        <v>25</v>
+        <v>146</v>
       </c>
       <c r="D57" t="s">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="E57">
-        <v>872143</v>
+        <v>877422</v>
       </c>
       <c r="F57" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="G57" t="s">
-        <v>86</v>
+        <v>59</v>
       </c>
       <c r="H57">
-        <v>6165.61</v>
+        <v>14815</v>
       </c>
       <c r="I57" s="1">
-        <v>46013.954583333303</v>
+        <v>46027.963391203702</v>
       </c>
       <c r="J57" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
@@ -2808,28 +2844,28 @@
         <v>148</v>
       </c>
       <c r="C58" t="s">
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="D58" t="s">
-        <v>99</v>
+        <v>40</v>
       </c>
       <c r="E58">
-        <v>872131</v>
+        <v>877951</v>
       </c>
       <c r="F58" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="G58" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="H58">
-        <v>13612</v>
+        <v>1901.83563237774</v>
       </c>
       <c r="I58" s="1">
-        <v>46013.9554166667</v>
+        <v>46027.964699074102</v>
       </c>
       <c r="J58" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
@@ -2837,31 +2873,31 @@
         <v>11</v>
       </c>
       <c r="B59" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="C59" t="s">
-        <v>136</v>
+        <v>107</v>
       </c>
       <c r="D59" t="s">
-        <v>137</v>
+        <v>108</v>
       </c>
       <c r="E59">
-        <v>861895</v>
+        <v>878142</v>
       </c>
       <c r="F59" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="G59" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="H59">
-        <v>5158.41</v>
+        <v>18572.0829015544</v>
       </c>
       <c r="I59" s="1">
-        <v>46013.969849537003</v>
+        <v>46028.0242939815</v>
       </c>
       <c r="J59" t="s">
-        <v>90</v>
+        <v>149</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
@@ -2869,28 +2905,28 @@
         <v>11</v>
       </c>
       <c r="B60" t="s">
-        <v>111</v>
+        <v>150</v>
       </c>
       <c r="C60" t="s">
-        <v>112</v>
+        <v>53</v>
       </c>
       <c r="D60" t="s">
-        <v>113</v>
+        <v>54</v>
       </c>
       <c r="E60">
-        <v>872046</v>
+        <v>878168</v>
       </c>
       <c r="F60" t="s">
-        <v>69</v>
+        <v>151</v>
       </c>
       <c r="G60" t="s">
-        <v>70</v>
+        <v>152</v>
       </c>
       <c r="H60">
-        <v>7015.94</v>
+        <v>5204.3261157024999</v>
       </c>
       <c r="I60" s="1">
-        <v>46014.051284722198</v>
+        <v>46028.035162036998</v>
       </c>
       <c r="J60" t="s">
         <v>149</v>
@@ -2901,28 +2937,28 @@
         <v>11</v>
       </c>
       <c r="B61" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C61" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D61" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E61">
-        <v>860925</v>
+        <v>877463</v>
       </c>
       <c r="F61" t="s">
-        <v>153</v>
+        <v>29</v>
       </c>
       <c r="G61" t="s">
-        <v>154</v>
+        <v>30</v>
       </c>
       <c r="H61">
-        <v>6330</v>
+        <v>2724.1438420107702</v>
       </c>
       <c r="I61" s="1">
-        <v>46014.055775462999</v>
+        <v>46028.054363425901</v>
       </c>
       <c r="J61" t="s">
         <v>149</v>
@@ -2933,28 +2969,28 @@
         <v>11</v>
       </c>
       <c r="B62" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C62" t="s">
-        <v>98</v>
+        <v>157</v>
       </c>
       <c r="D62" t="s">
-        <v>99</v>
+        <v>158</v>
       </c>
       <c r="E62">
-        <v>865002</v>
+        <v>863668</v>
       </c>
       <c r="F62" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="G62" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="H62">
-        <v>13044.29</v>
+        <v>13453</v>
       </c>
       <c r="I62" s="1">
-        <v>46014.082407407397</v>
+        <v>46028.063344907401</v>
       </c>
       <c r="J62" t="s">
         <v>149</v>
@@ -2965,28 +3001,28 @@
         <v>11</v>
       </c>
       <c r="B63" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C63" t="s">
-        <v>13</v>
+        <v>160</v>
       </c>
       <c r="D63" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="E63">
-        <v>862151</v>
+        <v>877540</v>
       </c>
       <c r="F63" t="s">
-        <v>15</v>
+        <v>142</v>
       </c>
       <c r="G63" t="s">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="H63">
-        <v>1623.62701600526</v>
+        <v>4411.7647058823504</v>
       </c>
       <c r="I63" s="1">
-        <v>46014.082719907397</v>
+        <v>46028.064039351899</v>
       </c>
       <c r="J63" t="s">
         <v>149</v>
@@ -2997,28 +3033,28 @@
         <v>11</v>
       </c>
       <c r="B64" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C64" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D64" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="E64">
-        <v>871275</v>
+        <v>877531</v>
       </c>
       <c r="F64" t="s">
-        <v>50</v>
+        <v>163</v>
       </c>
       <c r="G64" t="s">
-        <v>51</v>
+        <v>164</v>
       </c>
       <c r="H64">
-        <v>11918</v>
+        <v>6834</v>
       </c>
       <c r="I64" s="1">
-        <v>46014.099722222199</v>
+        <v>46028.080208333296</v>
       </c>
       <c r="J64" t="s">
         <v>149</v>
@@ -3029,28 +3065,28 @@
         <v>11</v>
       </c>
       <c r="B65" t="s">
-        <v>111</v>
+        <v>145</v>
       </c>
       <c r="C65" t="s">
-        <v>112</v>
+        <v>146</v>
       </c>
       <c r="D65" t="s">
-        <v>113</v>
+        <v>147</v>
       </c>
       <c r="E65">
-        <v>869261</v>
+        <v>877406</v>
       </c>
       <c r="F65" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="G65" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="H65">
-        <v>7015.94</v>
+        <v>5700.3</v>
       </c>
       <c r="I65" s="1">
-        <v>46014.104490740698</v>
+        <v>46028.116168981498</v>
       </c>
       <c r="J65" t="s">
         <v>149</v>
@@ -3061,28 +3097,28 @@
         <v>11</v>
       </c>
       <c r="B66" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="C66" t="s">
-        <v>35</v>
+        <v>98</v>
       </c>
       <c r="D66" t="s">
-        <v>36</v>
+        <v>99</v>
       </c>
       <c r="E66">
-        <v>864636</v>
+        <v>865567</v>
       </c>
       <c r="F66" t="s">
-        <v>27</v>
+        <v>166</v>
       </c>
       <c r="G66" t="s">
-        <v>28</v>
+        <v>167</v>
       </c>
       <c r="H66">
-        <v>12544</v>
+        <v>5556</v>
       </c>
       <c r="I66" s="1">
-        <v>46014.127638888902</v>
+        <v>46028.116990740702</v>
       </c>
       <c r="J66" t="s">
         <v>149</v>
@@ -3093,28 +3129,28 @@
         <v>11</v>
       </c>
       <c r="B67" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C67" t="s">
-        <v>159</v>
+        <v>39</v>
       </c>
       <c r="D67" t="s">
-        <v>160</v>
+        <v>40</v>
       </c>
       <c r="E67">
-        <v>872892</v>
+        <v>877058</v>
       </c>
       <c r="F67" t="s">
-        <v>106</v>
+        <v>168</v>
       </c>
       <c r="G67" t="s">
-        <v>107</v>
+        <v>169</v>
       </c>
       <c r="H67">
-        <v>11323.8</v>
+        <v>1816.11563237774</v>
       </c>
       <c r="I67" s="1">
-        <v>46014.134143518502</v>
+        <v>46028.118287037003</v>
       </c>
       <c r="J67" t="s">
         <v>149</v>
@@ -3125,28 +3161,28 @@
         <v>11</v>
       </c>
       <c r="B68" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C68" t="s">
-        <v>39</v>
+        <v>154</v>
       </c>
       <c r="D68" t="s">
-        <v>40</v>
+        <v>155</v>
       </c>
       <c r="E68">
-        <v>869270</v>
+        <v>877467</v>
       </c>
       <c r="F68" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="G68" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="H68">
-        <v>8823.15</v>
+        <v>2722.0238420107698</v>
       </c>
       <c r="I68" s="1">
-        <v>46014.134756944397</v>
+        <v>46028.119247685201</v>
       </c>
       <c r="J68" t="s">
         <v>149</v>
@@ -3157,28 +3193,28 @@
         <v>11</v>
       </c>
       <c r="B69" t="s">
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="C69" t="s">
-        <v>19</v>
+        <v>107</v>
       </c>
       <c r="D69" t="s">
-        <v>20</v>
+        <v>108</v>
       </c>
       <c r="E69">
-        <v>872773</v>
+        <v>878180</v>
       </c>
       <c r="F69" t="s">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="G69" t="s">
-        <v>22</v>
+        <v>77</v>
       </c>
       <c r="H69">
-        <v>10618</v>
+        <v>16150.0629015544</v>
       </c>
       <c r="I69" s="1">
-        <v>46014.1379282407</v>
+        <v>46028.120081018496</v>
       </c>
       <c r="J69" t="s">
         <v>149</v>
@@ -3189,28 +3225,28 @@
         <v>11</v>
       </c>
       <c r="B70" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C70" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="D70" t="s">
-        <v>133</v>
+        <v>40</v>
       </c>
       <c r="E70">
-        <v>872910</v>
+        <v>877058</v>
       </c>
       <c r="F70" t="s">
-        <v>95</v>
+        <v>168</v>
       </c>
       <c r="G70" t="s">
-        <v>96</v>
+        <v>169</v>
       </c>
       <c r="H70">
-        <v>1273.74999999999</v>
+        <v>9055.0999494097832</v>
       </c>
       <c r="I70" s="1">
-        <v>46014.1382407407</v>
+        <v>46028.131666666697</v>
       </c>
       <c r="J70" t="s">
         <v>149</v>
@@ -3221,28 +3257,28 @@
         <v>11</v>
       </c>
       <c r="B71" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="C71" t="s">
-        <v>32</v>
+        <v>114</v>
       </c>
       <c r="D71" t="s">
-        <v>33</v>
+        <v>115</v>
       </c>
       <c r="E71">
-        <v>871929</v>
+        <v>877734</v>
       </c>
       <c r="F71" t="s">
-        <v>163</v>
+        <v>36</v>
       </c>
       <c r="G71" t="s">
-        <v>164</v>
+        <v>37</v>
       </c>
       <c r="H71">
-        <v>7544.1</v>
+        <v>8144.3309248554997</v>
       </c>
       <c r="I71" s="1">
-        <v>46014.142326388901</v>
+        <v>46028.132581018501</v>
       </c>
       <c r="J71" t="s">
         <v>149</v>
@@ -3253,28 +3289,28 @@
         <v>11</v>
       </c>
       <c r="B72" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C72" t="s">
-        <v>132</v>
+        <v>172</v>
       </c>
       <c r="D72" t="s">
-        <v>133</v>
+        <v>173</v>
       </c>
       <c r="E72">
-        <v>872910</v>
+        <v>867972</v>
       </c>
       <c r="F72" t="s">
-        <v>95</v>
+        <v>174</v>
       </c>
       <c r="G72" t="s">
-        <v>96</v>
+        <v>175</v>
       </c>
       <c r="H72">
-        <v>15157</v>
+        <v>5700.57581573896</v>
       </c>
       <c r="I72" s="1">
-        <v>46014.164189814801</v>
+        <v>46028.133136574099</v>
       </c>
       <c r="J72" t="s">
         <v>149</v>
@@ -3285,28 +3321,28 @@
         <v>11</v>
       </c>
       <c r="B73" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="C73" t="s">
-        <v>32</v>
+        <v>122</v>
       </c>
       <c r="D73" t="s">
-        <v>33</v>
+        <v>123</v>
       </c>
       <c r="E73">
-        <v>871950</v>
+        <v>841390</v>
       </c>
       <c r="F73" t="s">
-        <v>127</v>
+        <v>78</v>
       </c>
       <c r="G73" t="s">
-        <v>128</v>
+        <v>79</v>
       </c>
       <c r="H73">
-        <v>14716</v>
+        <v>7224.0802675585301</v>
       </c>
       <c r="I73" s="1">
-        <v>46014.166631944398</v>
+        <v>46028.145023148201</v>
       </c>
       <c r="J73" t="s">
         <v>149</v>
@@ -3317,28 +3353,28 @@
         <v>11</v>
       </c>
       <c r="B74" t="s">
-        <v>38</v>
+        <v>177</v>
       </c>
       <c r="C74" t="s">
-        <v>39</v>
+        <v>178</v>
       </c>
       <c r="D74" t="s">
-        <v>40</v>
+        <v>179</v>
       </c>
       <c r="E74">
-        <v>871946</v>
+        <v>878085</v>
       </c>
       <c r="F74" t="s">
+        <v>65</v>
+      </c>
+      <c r="G74" t="s">
         <v>66</v>
       </c>
-      <c r="G74" t="s">
-        <v>67</v>
-      </c>
       <c r="H74">
-        <v>6543.26</v>
+        <v>5276</v>
       </c>
       <c r="I74" s="1">
-        <v>46014.208159722199</v>
+        <v>46028.150659722203</v>
       </c>
       <c r="J74" t="s">
         <v>149</v>
@@ -3349,28 +3385,28 @@
         <v>11</v>
       </c>
       <c r="B75" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="C75" t="s">
-        <v>168</v>
+        <v>107</v>
       </c>
       <c r="D75" t="s">
-        <v>169</v>
+        <v>108</v>
       </c>
       <c r="E75">
-        <v>872750</v>
+        <v>878147</v>
       </c>
       <c r="F75" t="s">
-        <v>170</v>
+        <v>76</v>
       </c>
       <c r="G75" t="s">
-        <v>171</v>
+        <v>77</v>
       </c>
       <c r="H75">
-        <v>10652</v>
+        <v>15536.8029015544</v>
       </c>
       <c r="I75" s="1">
-        <v>46014.214722222197</v>
+        <v>46028.151296296302</v>
       </c>
       <c r="J75" t="s">
         <v>149</v>
@@ -3381,28 +3417,28 @@
         <v>11</v>
       </c>
       <c r="B76" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C76" t="s">
-        <v>25</v>
+        <v>181</v>
       </c>
       <c r="D76" t="s">
-        <v>26</v>
+        <v>182</v>
       </c>
       <c r="E76">
-        <v>872150</v>
+        <v>874127</v>
       </c>
       <c r="F76" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="G76" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="H76">
-        <v>2059.4</v>
+        <v>4277</v>
       </c>
       <c r="I76" s="1">
-        <v>46014.2156944444</v>
+        <v>46028.177824074097</v>
       </c>
       <c r="J76" t="s">
         <v>149</v>
@@ -3413,28 +3449,28 @@
         <v>11</v>
       </c>
       <c r="B77" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="C77" t="s">
-        <v>13</v>
+        <v>98</v>
       </c>
       <c r="D77" t="s">
-        <v>14</v>
+        <v>99</v>
       </c>
       <c r="E77">
-        <v>862151</v>
+        <v>874127</v>
       </c>
       <c r="F77" t="s">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G77" t="s">
-        <v>16</v>
+        <v>101</v>
       </c>
       <c r="H77">
-        <v>2047.7307607980699</v>
+        <v>3372</v>
       </c>
       <c r="I77" s="1">
-        <v>46014.216099537</v>
+        <v>46028.187615740702</v>
       </c>
       <c r="J77" t="s">
         <v>149</v>
@@ -3445,28 +3481,28 @@
         <v>11</v>
       </c>
       <c r="B78" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="C78" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D78" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E78">
-        <v>862151</v>
+        <v>873095</v>
       </c>
       <c r="F78" t="s">
-        <v>15</v>
+        <v>163</v>
       </c>
       <c r="G78" t="s">
-        <v>16</v>
+        <v>164</v>
       </c>
       <c r="H78">
-        <v>1620.24</v>
+        <v>3572</v>
       </c>
       <c r="I78" s="1">
-        <v>46014.216296296298</v>
+        <v>46028.223842592597</v>
       </c>
       <c r="J78" t="s">
         <v>149</v>
@@ -3477,28 +3513,28 @@
         <v>11</v>
       </c>
       <c r="B79" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="C79" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="D79" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="E79">
-        <v>872915</v>
+        <v>877540</v>
       </c>
       <c r="F79" t="s">
-        <v>13</v>
+        <v>142</v>
       </c>
       <c r="G79" t="s">
-        <v>14</v>
+        <v>143</v>
       </c>
       <c r="H79">
-        <v>5730</v>
+        <v>11213.2352941176</v>
       </c>
       <c r="I79" s="1">
-        <v>46014.2656712963</v>
+        <v>46028.224409722199</v>
       </c>
       <c r="J79" t="s">
         <v>149</v>
@@ -3509,28 +3545,28 @@
         <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>178</v>
+        <v>144</v>
       </c>
       <c r="C80" t="s">
-        <v>179</v>
+        <v>107</v>
       </c>
       <c r="D80" t="s">
-        <v>180</v>
+        <v>108</v>
       </c>
       <c r="E80">
-        <v>865551</v>
+        <v>878185</v>
       </c>
       <c r="F80" t="s">
-        <v>181</v>
+        <v>76</v>
       </c>
       <c r="G80" t="s">
-        <v>182</v>
+        <v>77</v>
       </c>
       <c r="H80">
-        <v>7141.96</v>
+        <v>13198.502901554401</v>
       </c>
       <c r="I80" s="1">
-        <v>46014.302268518499</v>
+        <v>46028.224861111099</v>
       </c>
       <c r="J80" t="s">
         <v>149</v>
@@ -3541,30 +3577,382 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>183</v>
+        <v>153</v>
       </c>
       <c r="C81" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="D81" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="E81">
-        <v>872854</v>
+        <v>877463</v>
       </c>
       <c r="F81" t="s">
-        <v>122</v>
+        <v>29</v>
       </c>
       <c r="G81" t="s">
-        <v>123</v>
+        <v>30</v>
       </c>
       <c r="H81">
-        <v>18993</v>
+        <v>2039.12384201077</v>
       </c>
       <c r="I81" s="1">
-        <v>46014.314097222203</v>
+        <v>46028.225821759297</v>
       </c>
       <c r="J81" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>11</v>
+      </c>
+      <c r="B82" t="s">
+        <v>186</v>
+      </c>
+      <c r="C82" t="s">
+        <v>43</v>
+      </c>
+      <c r="D82" t="s">
+        <v>44</v>
+      </c>
+      <c r="E82">
+        <v>877495</v>
+      </c>
+      <c r="F82" t="s">
+        <v>130</v>
+      </c>
+      <c r="G82" t="s">
+        <v>131</v>
+      </c>
+      <c r="H82">
+        <v>9012</v>
+      </c>
+      <c r="I82" s="1">
+        <v>46028.226377314801</v>
+      </c>
+      <c r="J82" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>11</v>
+      </c>
+      <c r="B83" t="s">
+        <v>80</v>
+      </c>
+      <c r="C83" t="s">
+        <v>81</v>
+      </c>
+      <c r="D83" t="s">
+        <v>82</v>
+      </c>
+      <c r="E83">
+        <v>878202</v>
+      </c>
+      <c r="F83" t="s">
+        <v>83</v>
+      </c>
+      <c r="G83" t="s">
+        <v>84</v>
+      </c>
+      <c r="H83">
+        <v>15908.3873553719</v>
+      </c>
+      <c r="I83" s="1">
+        <v>46028.227997685201</v>
+      </c>
+      <c r="J83" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>11</v>
+      </c>
+      <c r="B84" t="s">
+        <v>171</v>
+      </c>
+      <c r="C84" t="s">
+        <v>172</v>
+      </c>
+      <c r="D84" t="s">
+        <v>173</v>
+      </c>
+      <c r="E84">
+        <v>872491</v>
+      </c>
+      <c r="F84" t="s">
+        <v>187</v>
+      </c>
+      <c r="G84" t="s">
+        <v>188</v>
+      </c>
+      <c r="H84">
+        <v>2821.2958157389598</v>
+      </c>
+      <c r="I84" s="1">
+        <v>46028.2346412037</v>
+      </c>
+      <c r="J84" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>11</v>
+      </c>
+      <c r="B85" t="s">
+        <v>189</v>
+      </c>
+      <c r="C85" t="s">
+        <v>157</v>
+      </c>
+      <c r="D85" t="s">
+        <v>158</v>
+      </c>
+      <c r="E85">
+        <v>841399</v>
+      </c>
+      <c r="F85" t="s">
+        <v>78</v>
+      </c>
+      <c r="G85" t="s">
+        <v>79</v>
+      </c>
+      <c r="H85">
+        <v>17489</v>
+      </c>
+      <c r="I85" s="1">
+        <v>46028.237268518496</v>
+      </c>
+      <c r="J85" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>11</v>
+      </c>
+      <c r="B86" t="s">
+        <v>190</v>
+      </c>
+      <c r="C86" t="s">
+        <v>191</v>
+      </c>
+      <c r="D86" t="s">
+        <v>192</v>
+      </c>
+      <c r="E86">
+        <v>868366</v>
+      </c>
+      <c r="F86" t="s">
+        <v>76</v>
+      </c>
+      <c r="G86" t="s">
+        <v>77</v>
+      </c>
+      <c r="H86">
+        <v>12954</v>
+      </c>
+      <c r="I86" s="1">
+        <v>46028.2495023148</v>
+      </c>
+      <c r="J86" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>11</v>
+      </c>
+      <c r="B87" t="s">
+        <v>193</v>
+      </c>
+      <c r="C87" t="s">
+        <v>107</v>
+      </c>
+      <c r="D87" t="s">
+        <v>108</v>
+      </c>
+      <c r="E87">
+        <v>864139</v>
+      </c>
+      <c r="F87" t="s">
+        <v>76</v>
+      </c>
+      <c r="G87" t="s">
+        <v>77</v>
+      </c>
+      <c r="H87">
+        <v>4455.9585492227998</v>
+      </c>
+      <c r="I87" s="1">
+        <v>46028.25</v>
+      </c>
+      <c r="J87" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>11</v>
+      </c>
+      <c r="B88" t="s">
+        <v>162</v>
+      </c>
+      <c r="C88" t="s">
+        <v>21</v>
+      </c>
+      <c r="D88" t="s">
+        <v>22</v>
+      </c>
+      <c r="E88">
+        <v>877490</v>
+      </c>
+      <c r="F88" t="s">
+        <v>163</v>
+      </c>
+      <c r="G88" t="s">
+        <v>164</v>
+      </c>
+      <c r="H88">
+        <v>1652.16</v>
+      </c>
+      <c r="I88" s="1">
+        <v>46028.263819444401</v>
+      </c>
+      <c r="J88" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>11</v>
+      </c>
+      <c r="B89" t="s">
+        <v>194</v>
+      </c>
+      <c r="C89" t="s">
+        <v>181</v>
+      </c>
+      <c r="D89" t="s">
+        <v>182</v>
+      </c>
+      <c r="E89">
+        <v>865567</v>
+      </c>
+      <c r="F89" t="s">
+        <v>166</v>
+      </c>
+      <c r="G89" t="s">
+        <v>167</v>
+      </c>
+      <c r="H89">
+        <v>4006</v>
+      </c>
+      <c r="I89" s="1">
+        <v>46028.302349537</v>
+      </c>
+      <c r="J89" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>11</v>
+      </c>
+      <c r="B90" t="s">
+        <v>165</v>
+      </c>
+      <c r="C90" t="s">
+        <v>98</v>
+      </c>
+      <c r="D90" t="s">
+        <v>99</v>
+      </c>
+      <c r="E90">
+        <v>874127</v>
+      </c>
+      <c r="F90" t="s">
+        <v>100</v>
+      </c>
+      <c r="G90" t="s">
+        <v>101</v>
+      </c>
+      <c r="H90">
+        <v>4730.2</v>
+      </c>
+      <c r="I90" s="1">
+        <v>46028.302916666697</v>
+      </c>
+      <c r="J90" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>11</v>
+      </c>
+      <c r="B91" t="s">
+        <v>195</v>
+      </c>
+      <c r="C91" t="s">
+        <v>107</v>
+      </c>
+      <c r="D91" t="s">
+        <v>108</v>
+      </c>
+      <c r="E91">
+        <v>864139</v>
+      </c>
+      <c r="F91" t="s">
+        <v>76</v>
+      </c>
+      <c r="G91" t="s">
+        <v>77</v>
+      </c>
+      <c r="H91">
+        <v>12279.792746114001</v>
+      </c>
+      <c r="I91" s="1">
+        <v>46028.303530092599</v>
+      </c>
+      <c r="J91" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>11</v>
+      </c>
+      <c r="B92" t="s">
+        <v>156</v>
+      </c>
+      <c r="C92" t="s">
+        <v>157</v>
+      </c>
+      <c r="D92" t="s">
+        <v>158</v>
+      </c>
+      <c r="E92">
+        <v>863681</v>
+      </c>
+      <c r="F92" t="s">
+        <v>78</v>
+      </c>
+      <c r="G92" t="s">
+        <v>79</v>
+      </c>
+      <c r="H92">
+        <v>12816.73</v>
+      </c>
+      <c r="I92" s="1">
+        <v>46028.3215740741</v>
+      </c>
+      <c r="J92" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>